<commit_message>
Overtime checker: add direct monthly work-site input
Add 입력_월별근무지 (same columns as the 365 monitoring workbook) so a
person's hospital for any month can be entered directly. Direct entries
take priority over the org list for the start/end-month hospitals of
month-crossing duties and for the target-month pay hospital, count as
being on the org list, and are labelled in a new 기관 출처 column.
Invalid month input now shows a text marker instead of #VALUE! in both
workbooks.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019ESd2Q14xCK8rv534PVGh3
</commit_message>
<xml_diff>
--- a/전공의_파견_모니터링_365.xlsx
+++ b/전공의_파견_모니터링_365.xlsx
@@ -625,13 +625,13 @@
     <tableColumn id="4" name="급여지급병원"/>
     <tableColumn id="5" name="비고"/>
     <tableColumn id="6" name="월키">
-      <calculatedColumnFormula>_xlfn.LET(_xlpm.v_m,월별근무지표[[#This Row],[월]],IF(_xlpm.v_m&amp;""="","",IF(ISNUMBER(_xlpm.v_m),IF(_xlpm.v_m&lt;10000,TEXT(DATE(INT(_xlpm.v_m),ROUND(MOD(_xlpm.v_m,1)*100,0),1),"yyyy-mm"),TEXT(_xlpm.v_m,"yyyy-mm")),TEXT(DATEVALUE(SUBSTITUTE(SUBSTITUTE(LEFT(TRIM(_xlpm.v_m),7),".","-"),"/","-")&amp;"-01"),"yyyy-mm"))))</calculatedColumnFormula>
+      <calculatedColumnFormula>_xlfn.LET(_xlpm.v_m,월별근무지표[[#This Row],[월]],IF(_xlpm.v_m&amp;""="","",IF(ISNUMBER(_xlpm.v_m),IF(_xlpm.v_m&lt;10000,TEXT(DATE(INT(_xlpm.v_m),ROUND(MOD(_xlpm.v_m,1)*100,0),1),"yyyy-mm"),TEXT(_xlpm.v_m,"yyyy-mm")),IFERROR(TEXT(DATEVALUE(SUBSTITUTE(SUBSTITUTE(LEFT(TRIM(_xlpm.v_m),7),".","-"),"/","-")&amp;"-01"),"yyyy-mm"),"⚠형식 오류"))))</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="7" name="사번키">
       <calculatedColumnFormula>IF(TRIM(월별근무지표[[#This Row],[사번]]&amp;"")="","","S|"&amp;TRIM(월별근무지표[[#This Row],[사번]]&amp;""))</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="8" name="키">
-      <calculatedColumnFormula>IF(ISERROR(월별근무지표[[#This Row],[월키]]),"",IF(OR(월별근무지표[[#This Row],[사번키]]="",월별근무지표[[#This Row],[월키]]=""),"",월별근무지표[[#This Row],[사번키]]&amp;"|"&amp;월별근무지표[[#This Row],[월키]]))</calculatedColumnFormula>
+      <calculatedColumnFormula>IF(LEFT(월별근무지표[[#This Row],[월키]],1)="⚠","",IF(OR(월별근무지표[[#This Row],[사번키]]="",월별근무지표[[#This Row],[월키]]=""),"",월별근무지표[[#This Row],[사번키]]&amp;"|"&amp;월별근무지표[[#This Row],[월키]]))</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="9" name="이름(확인)">
       <calculatedColumnFormula>IF(월별근무지표[[#This Row],[사번키]]="","",_xlfn.XLOOKUP(월별근무지표[[#This Row],[사번키]],기본자료표[사번키],기본자료표[이름]&amp;"","(기본자료에 없음)"))</calculatedColumnFormula>
@@ -640,7 +640,7 @@
       <calculatedColumnFormula>IF(월별근무지표[[#This Row],[근무병원]]="","",IF(월별근무지표[[#This Row],[급여지급병원]]="",월별근무지표[[#This Row],[근무병원]],월별근무지표[[#This Row],[급여지급병원]]))</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="11" name="점검">
-      <calculatedColumnFormula>IF(AND(TRIM(월별근무지표[[#This Row],[사번]]&amp;"")="",월별근무지표[[#This Row],[월]]&amp;""=""),"",IF(OR(TRIM(월별근무지표[[#This Row],[사번]]&amp;"")="",월별근무지표[[#This Row],[월]]&amp;""=""),"월·사번 모두 입력",IF(ISERROR(월별근무지표[[#This Row],[월키]]),"월 형식 확인(예: 2026-10)",IF(월별근무지표[[#This Row],[근무병원]]="","근무병원 입력",IF(COUNTIF(명단표[사번],TRIM(월별근무지표[[#This Row],[사번]]&amp;""))=0,"전공의명단에 없는 사번",IF(COUNTIF(월별근무지표[키],월별근무지표[[#This Row],[키]])&gt;1,"같은 사번·월 중복(위쪽 줄 적용)","정상"))))))</calculatedColumnFormula>
+      <calculatedColumnFormula>IF(AND(TRIM(월별근무지표[[#This Row],[사번]]&amp;"")="",월별근무지표[[#This Row],[월]]&amp;""=""),"",IF(OR(TRIM(월별근무지표[[#This Row],[사번]]&amp;"")="",월별근무지표[[#This Row],[월]]&amp;""=""),"월·사번 모두 입력",IF(LEFT(월별근무지표[[#This Row],[월키]],1)="⚠","월 형식 확인(예: 2026-10)",IF(월별근무지표[[#This Row],[근무병원]]="","근무병원 입력",IF(COUNTIF(명단표[사번],TRIM(월별근무지표[[#This Row],[사번]]&amp;""))=0,"전공의명단에 없는 사번",IF(COUNTIF(월별근무지표[키],월별근무지표[[#This Row],[키]])&gt;1,"같은 사번·월 중복(위쪽 줄 적용)","정상"))))))</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showRowStripes="1"/>
@@ -6545,7 +6545,7 @@
         </is>
       </c>
       <c r="F4" s="8">
-        <f>_xlfn.LET(_xlpm.v_m,월별근무지표[[#This Row],[월]],IF(_xlpm.v_m&amp;""="","",IF(ISNUMBER(_xlpm.v_m),IF(_xlpm.v_m&lt;10000,TEXT(DATE(INT(_xlpm.v_m),ROUND(MOD(_xlpm.v_m,1)*100,0),1),"yyyy-mm"),TEXT(_xlpm.v_m,"yyyy-mm")),TEXT(DATEVALUE(SUBSTITUTE(SUBSTITUTE(LEFT(TRIM(_xlpm.v_m),7),".","-"),"/","-")&amp;"-01"),"yyyy-mm"))))</f>
+        <f>_xlfn.LET(_xlpm.v_m,월별근무지표[[#This Row],[월]],IF(_xlpm.v_m&amp;""="","",IF(ISNUMBER(_xlpm.v_m),IF(_xlpm.v_m&lt;10000,TEXT(DATE(INT(_xlpm.v_m),ROUND(MOD(_xlpm.v_m,1)*100,0),1),"yyyy-mm"),TEXT(_xlpm.v_m,"yyyy-mm")),IFERROR(TEXT(DATEVALUE(SUBSTITUTE(SUBSTITUTE(LEFT(TRIM(_xlpm.v_m),7),".","-"),"/","-")&amp;"-01"),"yyyy-mm"),"⚠형식 오류"))))</f>
         <v/>
       </c>
       <c r="G4" s="8">
@@ -6553,7 +6553,7 @@
         <v/>
       </c>
       <c r="H4" s="8">
-        <f>IF(ISERROR(월별근무지표[[#This Row],[월키]]),"",IF(OR(월별근무지표[[#This Row],[사번키]]="",월별근무지표[[#This Row],[월키]]=""),"",월별근무지표[[#This Row],[사번키]]&amp;"|"&amp;월별근무지표[[#This Row],[월키]]))</f>
+        <f>IF(LEFT(월별근무지표[[#This Row],[월키]],1)="⚠","",IF(OR(월별근무지표[[#This Row],[사번키]]="",월별근무지표[[#This Row],[월키]]=""),"",월별근무지표[[#This Row],[사번키]]&amp;"|"&amp;월별근무지표[[#This Row],[월키]]))</f>
         <v/>
       </c>
       <c r="I4" s="8">
@@ -6565,7 +6565,7 @@
         <v/>
       </c>
       <c r="K4" s="8">
-        <f>IF(AND(TRIM(월별근무지표[[#This Row],[사번]]&amp;"")="",월별근무지표[[#This Row],[월]]&amp;""=""),"",IF(OR(TRIM(월별근무지표[[#This Row],[사번]]&amp;"")="",월별근무지표[[#This Row],[월]]&amp;""=""),"월·사번 모두 입력",IF(ISERROR(월별근무지표[[#This Row],[월키]]),"월 형식 확인(예: 2026-10)",IF(월별근무지표[[#This Row],[근무병원]]="","근무병원 입력",IF(COUNTIF(명단표[사번],TRIM(월별근무지표[[#This Row],[사번]]&amp;""))=0,"전공의명단에 없는 사번",IF(COUNTIF(월별근무지표[키],월별근무지표[[#This Row],[키]])&gt;1,"같은 사번·월 중복(위쪽 줄 적용)","정상"))))))</f>
+        <f>IF(AND(TRIM(월별근무지표[[#This Row],[사번]]&amp;"")="",월별근무지표[[#This Row],[월]]&amp;""=""),"",IF(OR(TRIM(월별근무지표[[#This Row],[사번]]&amp;"")="",월별근무지표[[#This Row],[월]]&amp;""=""),"월·사번 모두 입력",IF(LEFT(월별근무지표[[#This Row],[월키]],1)="⚠","월 형식 확인(예: 2026-10)",IF(월별근무지표[[#This Row],[근무병원]]="","근무병원 입력",IF(COUNTIF(명단표[사번],TRIM(월별근무지표[[#This Row],[사번]]&amp;""))=0,"전공의명단에 없는 사번",IF(COUNTIF(월별근무지표[키],월별근무지표[[#This Row],[키]])&gt;1,"같은 사번·월 중복(위쪽 줄 적용)","정상"))))))</f>
         <v/>
       </c>
     </row>
@@ -6590,7 +6590,7 @@
         </is>
       </c>
       <c r="F5" s="8">
-        <f>_xlfn.LET(_xlpm.v_m,월별근무지표[[#This Row],[월]],IF(_xlpm.v_m&amp;""="","",IF(ISNUMBER(_xlpm.v_m),IF(_xlpm.v_m&lt;10000,TEXT(DATE(INT(_xlpm.v_m),ROUND(MOD(_xlpm.v_m,1)*100,0),1),"yyyy-mm"),TEXT(_xlpm.v_m,"yyyy-mm")),TEXT(DATEVALUE(SUBSTITUTE(SUBSTITUTE(LEFT(TRIM(_xlpm.v_m),7),".","-"),"/","-")&amp;"-01"),"yyyy-mm"))))</f>
+        <f>_xlfn.LET(_xlpm.v_m,월별근무지표[[#This Row],[월]],IF(_xlpm.v_m&amp;""="","",IF(ISNUMBER(_xlpm.v_m),IF(_xlpm.v_m&lt;10000,TEXT(DATE(INT(_xlpm.v_m),ROUND(MOD(_xlpm.v_m,1)*100,0),1),"yyyy-mm"),TEXT(_xlpm.v_m,"yyyy-mm")),IFERROR(TEXT(DATEVALUE(SUBSTITUTE(SUBSTITUTE(LEFT(TRIM(_xlpm.v_m),7),".","-"),"/","-")&amp;"-01"),"yyyy-mm"),"⚠형식 오류"))))</f>
         <v/>
       </c>
       <c r="G5" s="8">
@@ -6598,7 +6598,7 @@
         <v/>
       </c>
       <c r="H5" s="8">
-        <f>IF(ISERROR(월별근무지표[[#This Row],[월키]]),"",IF(OR(월별근무지표[[#This Row],[사번키]]="",월별근무지표[[#This Row],[월키]]=""),"",월별근무지표[[#This Row],[사번키]]&amp;"|"&amp;월별근무지표[[#This Row],[월키]]))</f>
+        <f>IF(LEFT(월별근무지표[[#This Row],[월키]],1)="⚠","",IF(OR(월별근무지표[[#This Row],[사번키]]="",월별근무지표[[#This Row],[월키]]=""),"",월별근무지표[[#This Row],[사번키]]&amp;"|"&amp;월별근무지표[[#This Row],[월키]]))</f>
         <v/>
       </c>
       <c r="I5" s="8">
@@ -6610,7 +6610,7 @@
         <v/>
       </c>
       <c r="K5" s="8">
-        <f>IF(AND(TRIM(월별근무지표[[#This Row],[사번]]&amp;"")="",월별근무지표[[#This Row],[월]]&amp;""=""),"",IF(OR(TRIM(월별근무지표[[#This Row],[사번]]&amp;"")="",월별근무지표[[#This Row],[월]]&amp;""=""),"월·사번 모두 입력",IF(ISERROR(월별근무지표[[#This Row],[월키]]),"월 형식 확인(예: 2026-10)",IF(월별근무지표[[#This Row],[근무병원]]="","근무병원 입력",IF(COUNTIF(명단표[사번],TRIM(월별근무지표[[#This Row],[사번]]&amp;""))=0,"전공의명단에 없는 사번",IF(COUNTIF(월별근무지표[키],월별근무지표[[#This Row],[키]])&gt;1,"같은 사번·월 중복(위쪽 줄 적용)","정상"))))))</f>
+        <f>IF(AND(TRIM(월별근무지표[[#This Row],[사번]]&amp;"")="",월별근무지표[[#This Row],[월]]&amp;""=""),"",IF(OR(TRIM(월별근무지표[[#This Row],[사번]]&amp;"")="",월별근무지표[[#This Row],[월]]&amp;""=""),"월·사번 모두 입력",IF(LEFT(월별근무지표[[#This Row],[월키]],1)="⚠","월 형식 확인(예: 2026-10)",IF(월별근무지표[[#This Row],[근무병원]]="","근무병원 입력",IF(COUNTIF(명단표[사번],TRIM(월별근무지표[[#This Row],[사번]]&amp;""))=0,"전공의명단에 없는 사번",IF(COUNTIF(월별근무지표[키],월별근무지표[[#This Row],[키]])&gt;1,"같은 사번·월 중복(위쪽 줄 적용)","정상"))))))</f>
         <v/>
       </c>
     </row>
@@ -6639,7 +6639,7 @@
         </is>
       </c>
       <c r="F6" s="8">
-        <f>_xlfn.LET(_xlpm.v_m,월별근무지표[[#This Row],[월]],IF(_xlpm.v_m&amp;""="","",IF(ISNUMBER(_xlpm.v_m),IF(_xlpm.v_m&lt;10000,TEXT(DATE(INT(_xlpm.v_m),ROUND(MOD(_xlpm.v_m,1)*100,0),1),"yyyy-mm"),TEXT(_xlpm.v_m,"yyyy-mm")),TEXT(DATEVALUE(SUBSTITUTE(SUBSTITUTE(LEFT(TRIM(_xlpm.v_m),7),".","-"),"/","-")&amp;"-01"),"yyyy-mm"))))</f>
+        <f>_xlfn.LET(_xlpm.v_m,월별근무지표[[#This Row],[월]],IF(_xlpm.v_m&amp;""="","",IF(ISNUMBER(_xlpm.v_m),IF(_xlpm.v_m&lt;10000,TEXT(DATE(INT(_xlpm.v_m),ROUND(MOD(_xlpm.v_m,1)*100,0),1),"yyyy-mm"),TEXT(_xlpm.v_m,"yyyy-mm")),IFERROR(TEXT(DATEVALUE(SUBSTITUTE(SUBSTITUTE(LEFT(TRIM(_xlpm.v_m),7),".","-"),"/","-")&amp;"-01"),"yyyy-mm"),"⚠형식 오류"))))</f>
         <v/>
       </c>
       <c r="G6" s="8">
@@ -6647,7 +6647,7 @@
         <v/>
       </c>
       <c r="H6" s="8">
-        <f>IF(ISERROR(월별근무지표[[#This Row],[월키]]),"",IF(OR(월별근무지표[[#This Row],[사번키]]="",월별근무지표[[#This Row],[월키]]=""),"",월별근무지표[[#This Row],[사번키]]&amp;"|"&amp;월별근무지표[[#This Row],[월키]]))</f>
+        <f>IF(LEFT(월별근무지표[[#This Row],[월키]],1)="⚠","",IF(OR(월별근무지표[[#This Row],[사번키]]="",월별근무지표[[#This Row],[월키]]=""),"",월별근무지표[[#This Row],[사번키]]&amp;"|"&amp;월별근무지표[[#This Row],[월키]]))</f>
         <v/>
       </c>
       <c r="I6" s="8">
@@ -6659,7 +6659,7 @@
         <v/>
       </c>
       <c r="K6" s="8">
-        <f>IF(AND(TRIM(월별근무지표[[#This Row],[사번]]&amp;"")="",월별근무지표[[#This Row],[월]]&amp;""=""),"",IF(OR(TRIM(월별근무지표[[#This Row],[사번]]&amp;"")="",월별근무지표[[#This Row],[월]]&amp;""=""),"월·사번 모두 입력",IF(ISERROR(월별근무지표[[#This Row],[월키]]),"월 형식 확인(예: 2026-10)",IF(월별근무지표[[#This Row],[근무병원]]="","근무병원 입력",IF(COUNTIF(명단표[사번],TRIM(월별근무지표[[#This Row],[사번]]&amp;""))=0,"전공의명단에 없는 사번",IF(COUNTIF(월별근무지표[키],월별근무지표[[#This Row],[키]])&gt;1,"같은 사번·월 중복(위쪽 줄 적용)","정상"))))))</f>
+        <f>IF(AND(TRIM(월별근무지표[[#This Row],[사번]]&amp;"")="",월별근무지표[[#This Row],[월]]&amp;""=""),"",IF(OR(TRIM(월별근무지표[[#This Row],[사번]]&amp;"")="",월별근무지표[[#This Row],[월]]&amp;""=""),"월·사번 모두 입력",IF(LEFT(월별근무지표[[#This Row],[월키]],1)="⚠","월 형식 확인(예: 2026-10)",IF(월별근무지표[[#This Row],[근무병원]]="","근무병원 입력",IF(COUNTIF(명단표[사번],TRIM(월별근무지표[[#This Row],[사번]]&amp;""))=0,"전공의명단에 없는 사번",IF(COUNTIF(월별근무지표[키],월별근무지표[[#This Row],[키]])&gt;1,"같은 사번·월 중복(위쪽 줄 적용)","정상"))))))</f>
         <v/>
       </c>
     </row>

</xml_diff>